<commit_message>
depin: swap confirmed open - canon note, playbook AMM rule, sheet note
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014drgzQYBXTLjd1zzmsjRaS
</commit_message>
<xml_diff>
--- a/depin/content/ai-pass-compound-1016.xlsx
+++ b/depin/content/ai-pass-compound-1016.xlsx
@@ -4823,7 +4823,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">: </t>
+      <t xml:space="preserve">: 10/17 </t>
     </r>
     <r>
       <rPr>
@@ -4831,7 +4831,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">적립분이 계정 포인트로만 쌓이는 단계면</t>
+      <t xml:space="preserve">서우 확인 — 적립분은 바로 </t>
     </r>
     <r>
       <rPr>
@@ -4840,7 +4840,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">(FAQ </t>
+      <t xml:space="preserve">XRP · RLUSD </t>
     </r>
     <r>
       <rPr>
@@ -4848,7 +4848,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">「출금 개시 전 계정 포인트」</t>
+      <t xml:space="preserve">로 스왑된다</t>
     </r>
     <r>
       <rPr>
@@ -4857,7 +4857,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">) </t>
+      <t xml:space="preserve">. </t>
     </r>
     <r>
       <rPr>
@@ -4865,7 +4865,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">지갑으로 꺼내 팔 수 없다</t>
+      <t xml:space="preserve">남은 위험은 가격 영향뿐</t>
     </r>
     <r>
       <rPr>
@@ -4882,7 +4882,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">정본 </t>
+      <t xml:space="preserve">위 풀 깊이 계산</t>
     </r>
     <r>
       <rPr>
@@ -4891,7 +4891,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">§4-1 </t>
+      <t xml:space="preserve">) — </t>
     </r>
     <r>
       <rPr>
@@ -4899,7 +4899,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">확인 필요 ②</t>
+      <t xml:space="preserve">한 사람의 하루 적립은 영향이 거의 없지만</t>
     </r>
     <r>
       <rPr>
@@ -4908,7 +4908,24 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">).</t>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보유자 다수가 같은 날 팔면 풀 가격이 크게 밀린다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
     </r>
   </si>
   <si>

</xml_diff>